<commit_message>
Save all code on develop branch
</commit_message>
<xml_diff>
--- a/exports/visitors.xlsx
+++ b/exports/visitors.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
   <si>
     <t>ID</t>
   </si>
@@ -84,6 +84,18 @@
   </si>
   <si>
     <t>2026-06-08T13:14:21.885137</t>
+  </si>
+  <si>
+    <t>Ravi</t>
+  </si>
+  <si>
+    <t>9876543915</t>
+  </si>
+  <si>
+    <t>Rajesh@gmail.com</t>
+  </si>
+  <si>
+    <t>2026-06-08T16:12:19.070162</t>
   </si>
 </sst>
 </file>
@@ -134,7 +146,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="2.71875" customWidth="true" bestFit="true"/>
@@ -261,6 +273,29 @@
         <v>23</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="n" s="0">
+        <v>5.0</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>27</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Added email and mobile validation
</commit_message>
<xml_diff>
--- a/exports/visitors.xlsx
+++ b/exports/visitors.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="33">
   <si>
     <t>ID</t>
   </si>
@@ -35,6 +35,9 @@
     <t>Visit Time</t>
   </si>
   <si>
+    <t>PhotoURL</t>
+  </si>
+  <si>
     <t>Ravi Kumar</t>
   </si>
   <si>
@@ -53,6 +56,9 @@
     <t>2026-06-04T13:20:24.943653</t>
   </si>
   <si>
+    <t>https://cloudinary.com/images/photo1.jpg</t>
+  </si>
+  <si>
     <t>9876543910</t>
   </si>
   <si>
@@ -96,6 +102,15 @@
   </si>
   <si>
     <t>2026-06-08T16:12:19.070162</t>
+  </si>
+  <si>
+    <t>9876543916</t>
+  </si>
+  <si>
+    <t>Rajes@gmail.com</t>
+  </si>
+  <si>
+    <t>2026-06-10T09:51:24.170919</t>
   </si>
 </sst>
 </file>
@@ -146,7 +161,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="2.71875" customWidth="true" bestFit="true"/>
@@ -156,6 +171,7 @@
     <col min="5" max="5" width="10.03125" customWidth="true" bestFit="true"/>
     <col min="6" max="6" width="9.0234375" customWidth="true" bestFit="true"/>
     <col min="7" max="7" width="24.65234375" customWidth="true" bestFit="true"/>
+    <col min="8" max="8" width="35.4453125" customWidth="true" bestFit="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -180,28 +196,34 @@
       <c r="G1" t="s" s="1">
         <v>6</v>
       </c>
+      <c r="H1" t="s" s="1">
+        <v>7</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n" s="0">
         <v>1.0</v>
       </c>
       <c r="B2" t="s" s="0">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C2" t="s" s="0">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D2" t="s" s="0">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s" s="0">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F2" t="s" s="0">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G2" t="s" s="0">
-        <v>12</v>
+        <v>13</v>
+      </c>
+      <c r="H2" t="s" s="0">
+        <v>14</v>
       </c>
     </row>
     <row r="3">
@@ -209,22 +231,25 @@
         <v>2.0</v>
       </c>
       <c r="B3" t="s" s="0">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s" s="0">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G3" t="s" s="0">
-        <v>15</v>
+        <v>17</v>
+      </c>
+      <c r="H3" t="s" s="0">
+        <v>14</v>
       </c>
     </row>
     <row r="4">
@@ -232,22 +257,25 @@
         <v>3.0</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G4" t="s" s="0">
-        <v>19</v>
+        <v>21</v>
+      </c>
+      <c r="H4" t="s" s="0">
+        <v>14</v>
       </c>
     </row>
     <row r="5">
@@ -255,22 +283,25 @@
         <v>4.0</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G5" t="s" s="0">
-        <v>23</v>
+        <v>25</v>
+      </c>
+      <c r="H5" t="s" s="0">
+        <v>14</v>
       </c>
     </row>
     <row r="6">
@@ -278,22 +309,51 @@
         <v>5.0</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D6" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G6" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="H6" t="s" s="0">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n" s="0">
+        <v>7.0</v>
+      </c>
+      <c r="B7" t="s" s="0">
         <v>26</v>
       </c>
-      <c r="E6" t="s" s="0">
-        <v>10</v>
-      </c>
-      <c r="F6" t="s" s="0">
-        <v>11</v>
-      </c>
-      <c r="G6" t="s" s="0">
-        <v>27</v>
+      <c r="C7" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="G7" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="H7" t="s" s="0">
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>